<commit_message>
version 1 output file is correct
</commit_message>
<xml_diff>
--- a/outputs/modified_reservation.xlsx
+++ b/outputs/modified_reservation.xlsx
@@ -446,7 +446,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3000</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="3">
@@ -457,11 +457,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Gary</t>
+          <t>Chloe</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>5000</v>
+        <v>3000</v>
       </c>
     </row>
   </sheetData>
@@ -518,11 +518,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Chloe</t>
+          <t>Susan</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>6000</v>
+        <v>4000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Version 1.1.0 implemented autofit column feature
</commit_message>
<xml_diff>
--- a/outputs/modified_reservation.xlsx
+++ b/outputs/modified_reservation.xlsx
@@ -416,6 +416,11 @@
   </sheetPr>
   <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -477,6 +482,11 @@
   </sheetPr>
   <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">

</xml_diff>

<commit_message>
Version 1.2.0 Auto_Sum added!
</commit_message>
<xml_diff>
--- a/outputs/modified_reservation.xlsx
+++ b/outputs/modified_reservation.xlsx
@@ -9,6 +9,8 @@
   <sheets>
     <sheet name="agoda" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="booking.com" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="expedia" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="trip.com" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -467,6 +469,12 @@
       </c>
       <c r="C3" t="n">
         <v>3000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="C4">
+        <f>SUM(C2:C3)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -480,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -535,6 +543,156 @@
         <v>4000</v>
       </c>
     </row>
+    <row r="4">
+      <c r="C4">
+        <f>SUM(C2:C3)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>reservation site</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>guest name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>expedia</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Cho</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>expedia</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Matt</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="C4">
+        <f>SUM(C2:C3)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>reservation site</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>guest name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>trip.com</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Gary</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>trip.com</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Harry</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2100</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="C4">
+        <f>SUM(C2:C3)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
csv and xlxs both are supported v1.3.1
</commit_message>
<xml_diff>
--- a/outputs/modified_reservation.xlsx
+++ b/outputs/modified_reservation.xlsx
@@ -9,8 +9,6 @@
   <sheets>
     <sheet name="agoda" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="booking.com" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="expedia" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="trip.com" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -552,148 +550,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>reservation site</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>guest name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>amount</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>expedia</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Cho</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>expedia</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Matt</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="C4">
-        <f>SUM(C2:C3)</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>reservation site</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>guest name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>amount</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>trip.com</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Gary</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>1500</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>trip.com</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Harry</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>2100</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="C4">
-        <f>SUM(C2:C3)</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>